<commit_message>
Updating k6 scritps duration limits Upgrading to service-core 1.0.0-beta.5
</commit_message>
<xml_diff>
--- a/k6-tests/results.xlsx
+++ b/k6-tests/results.xlsx
@@ -8,12 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\github\rapidrest\petstore_example\k6-tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5D8B515-D5D8-4735-83E0-40997EFD59EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD175F35-4744-49B0-AD73-534B974D1F74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="270" yWindow="1155" windowWidth="24930" windowHeight="17985" xr2:uid="{FF28AC9A-F1E0-4B8D-AFDC-88670F014157}"/>
+    <workbookView xWindow="12705" yWindow="285" windowWidth="25215" windowHeight="18735" xr2:uid="{FF28AC9A-F1E0-4B8D-AFDC-88670F014157}"/>
   </bookViews>
   <sheets>
-    <sheet name="1.0.31-cjs" sheetId="1" r:id="rId1"/>
+    <sheet name="Comparison" sheetId="3" r:id="rId1"/>
+    <sheet name="1.0.31-rrst" sheetId="2" r:id="rId2"/>
+    <sheet name="1.0.31-cjs" sheetId="1" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,14 +38,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="26">
   <si>
     <t>Test</t>
   </si>
   <si>
-    <t>Req Failed</t>
-  </si>
-  <si>
     <t>Req/Sec</t>
   </si>
   <si>
@@ -68,12 +67,6 @@
     <t>Duration (p90)</t>
   </si>
   <si>
-    <t>Total Req</t>
-  </si>
-  <si>
-    <t>% Failed</t>
-  </si>
-  <si>
     <t>create_user</t>
   </si>
   <si>
@@ -90,15 +83,45 @@
   </si>
   <si>
     <t>find_pets</t>
+  </si>
+  <si>
+    <t>Perf Gain (Req/Sec)</t>
+  </si>
+  <si>
+    <t>Perf Gain (Avg)</t>
+  </si>
+  <si>
+    <t>Perf Gain (p90)</t>
+  </si>
+  <si>
+    <t>Perf Gain (p95)</t>
+  </si>
+  <si>
+    <t>Diff</t>
+  </si>
+  <si>
+    <t>Composer.js Req/Sec</t>
+  </si>
+  <si>
+    <t>RapidREST Req/Sec</t>
+  </si>
+  <si>
+    <t>Composer.js p90 (ms)</t>
+  </si>
+  <si>
+    <t>RapidREST p90 (ms)</t>
+  </si>
+  <si>
+    <t>Composer.js p95 (ms)</t>
+  </si>
+  <si>
+    <t>RapidREST p95 (ms)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="166" formatCode="0.0000%"/>
-  </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -144,10 +167,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -482,309 +506,951 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{059A8E8E-4130-4CCA-A3A8-A42D26512C95}">
-  <dimension ref="A1:K8"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5D097EAA-5212-49A2-BFBD-5BDD634282B9}">
+  <dimension ref="A1:L8"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="21" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="21" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="19.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2">
+        <f>'1.0.31-cjs'!C2</f>
+        <v>71.816000000000003</v>
+      </c>
+      <c r="C2">
+        <f>'1.0.31-rrst'!C2</f>
+        <v>70.688999999999993</v>
+      </c>
+      <c r="D2" s="3">
+        <f>(C2/B2)-1</f>
+        <v>-1.5692881809067805E-2</v>
+      </c>
+      <c r="F2">
+        <f>'1.0.31-cjs'!G2</f>
+        <v>1430</v>
+      </c>
+      <c r="G2">
+        <f>'1.0.31-rrst'!G2</f>
+        <v>1440</v>
+      </c>
+      <c r="H2" s="3">
+        <f>(F2/G2)-1</f>
+        <v>-6.9444444444444198E-3</v>
+      </c>
+      <c r="J2">
+        <f>'1.0.31-cjs'!H2</f>
+        <v>1490</v>
+      </c>
+      <c r="K2">
+        <f>'1.0.31-rrst'!H2</f>
+        <v>1460</v>
+      </c>
+      <c r="L2" s="3">
+        <f>(J2/K2)-1</f>
+        <v>2.0547945205479534E-2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3">
+        <f>'1.0.31-cjs'!C3</f>
+        <v>2058.9180000000001</v>
+      </c>
+      <c r="C3">
+        <f>'1.0.31-rrst'!C3</f>
+        <v>3673.1170000000002</v>
+      </c>
+      <c r="D3" s="3">
+        <f t="shared" ref="D3:D8" si="0">(C3/B3)-1</f>
+        <v>0.78400353972329162</v>
+      </c>
+      <c r="F3">
+        <f>'1.0.31-cjs'!G3</f>
+        <v>62.05</v>
+      </c>
+      <c r="G3">
+        <f>'1.0.31-rrst'!G3</f>
+        <v>36.130000000000003</v>
+      </c>
+      <c r="H3" s="3">
+        <f t="shared" ref="H3:H8" si="1">(F3/G3)-1</f>
+        <v>0.71740935510655945</v>
+      </c>
+      <c r="J3">
+        <f>'1.0.31-cjs'!H3</f>
+        <v>65.72</v>
+      </c>
+      <c r="K3">
+        <f>'1.0.31-rrst'!H3</f>
+        <v>37.97</v>
+      </c>
+      <c r="L3" s="3">
+        <f t="shared" ref="L3:L8" si="2">(J3/K3)-1</f>
+        <v>0.73084013695022398</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4">
+        <f>'1.0.31-cjs'!C4</f>
+        <v>5905.6930000000002</v>
+      </c>
+      <c r="C4">
+        <f>'1.0.31-rrst'!C4</f>
+        <v>9494.1419999999998</v>
+      </c>
+      <c r="D4" s="3">
+        <f t="shared" si="0"/>
+        <v>0.6076253879095983</v>
+      </c>
+      <c r="F4">
+        <f>'1.0.31-cjs'!G4</f>
+        <v>23.13</v>
+      </c>
+      <c r="G4">
+        <f>'1.0.31-rrst'!G4</f>
+        <v>14.62</v>
+      </c>
+      <c r="H4" s="3">
+        <f t="shared" si="1"/>
+        <v>0.58207934336525313</v>
+      </c>
+      <c r="J4">
+        <f>'1.0.31-cjs'!H4</f>
+        <v>24.24</v>
+      </c>
+      <c r="K4">
+        <f>'1.0.31-rrst'!H4</f>
+        <v>16.100000000000001</v>
+      </c>
+      <c r="L4" s="3">
+        <f t="shared" si="2"/>
+        <v>0.50559006211180102</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5">
+        <f>'1.0.31-cjs'!C5</f>
+        <v>2520.547</v>
+      </c>
+      <c r="C5">
+        <f>'1.0.31-rrst'!C5</f>
+        <v>4125.4129999999996</v>
+      </c>
+      <c r="D5" s="3">
+        <f t="shared" si="0"/>
+        <v>0.63671338007186518</v>
+      </c>
+      <c r="F5">
+        <f>'1.0.31-cjs'!G5</f>
+        <v>42.44</v>
+      </c>
+      <c r="G5">
+        <f>'1.0.31-rrst'!G5</f>
+        <v>38.049999999999997</v>
+      </c>
+      <c r="H5" s="3">
+        <f t="shared" si="1"/>
+        <v>0.11537450722733245</v>
+      </c>
+      <c r="J5">
+        <f>'1.0.31-cjs'!H5</f>
+        <v>43.81</v>
+      </c>
+      <c r="K5">
+        <f>'1.0.31-rrst'!H5</f>
+        <v>41.97</v>
+      </c>
+      <c r="L5" s="3">
+        <f t="shared" si="2"/>
+        <v>4.384083869430544E-2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6">
+        <f>'1.0.31-cjs'!C6</f>
+        <v>187.39500000000001</v>
+      </c>
+      <c r="C6">
+        <f>'1.0.31-rrst'!C6</f>
+        <v>217.511</v>
+      </c>
+      <c r="D6" s="3">
+        <f t="shared" si="0"/>
+        <v>0.16070866351823687</v>
+      </c>
+      <c r="F6">
+        <f>'1.0.31-cjs'!G6</f>
+        <v>585.67999999999995</v>
+      </c>
+      <c r="G6">
+        <f>'1.0.31-rrst'!G6</f>
+        <v>474.76</v>
+      </c>
+      <c r="H6" s="3">
+        <f t="shared" si="1"/>
+        <v>0.23363383604347443</v>
+      </c>
+      <c r="J6">
+        <f>'1.0.31-cjs'!H6</f>
+        <v>622.70000000000005</v>
+      </c>
+      <c r="K6">
+        <f>'1.0.31-rrst'!H6</f>
+        <v>484.99</v>
+      </c>
+      <c r="L6" s="3">
+        <f t="shared" si="2"/>
+        <v>0.28394399884533716</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7">
+        <f>'1.0.31-cjs'!C7</f>
+        <v>4093.308</v>
+      </c>
+      <c r="C7">
+        <f>'1.0.31-rrst'!C7</f>
+        <v>7643.0460000000003</v>
+      </c>
+      <c r="D7" s="3">
+        <f t="shared" si="0"/>
+        <v>0.86720520420158964</v>
+      </c>
+      <c r="F7">
+        <f>'1.0.31-cjs'!G7</f>
+        <v>30.24</v>
+      </c>
+      <c r="G7">
+        <f>'1.0.31-rrst'!G7</f>
+        <v>17.63</v>
+      </c>
+      <c r="H7" s="3">
+        <f t="shared" si="1"/>
+        <v>0.71525808281338632</v>
+      </c>
+      <c r="J7">
+        <f>'1.0.31-cjs'!H7</f>
+        <v>33.46</v>
+      </c>
+      <c r="K7">
+        <f>'1.0.31-rrst'!H7</f>
+        <v>19.28</v>
+      </c>
+      <c r="L7" s="3">
+        <f t="shared" si="2"/>
+        <v>0.73547717842323657</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8">
+        <f>'1.0.31-cjs'!C8</f>
+        <v>70.126999999999995</v>
+      </c>
+      <c r="C8">
+        <f>'1.0.31-rrst'!C8</f>
+        <v>70.218999999999994</v>
+      </c>
+      <c r="D8" s="3">
+        <f t="shared" si="0"/>
+        <v>1.3119055428008064E-3</v>
+      </c>
+      <c r="F8">
+        <f>'1.0.31-cjs'!G8</f>
+        <v>1450</v>
+      </c>
+      <c r="G8">
+        <f>'1.0.31-rrst'!G8</f>
+        <v>1440</v>
+      </c>
+      <c r="H8" s="3">
+        <f t="shared" si="1"/>
+        <v>6.9444444444444198E-3</v>
+      </c>
+      <c r="J8">
+        <f>'1.0.31-cjs'!H8</f>
+        <v>1470</v>
+      </c>
+      <c r="K8">
+        <f>'1.0.31-rrst'!H8</f>
+        <v>1450</v>
+      </c>
+      <c r="L8" s="3">
+        <f t="shared" si="2"/>
+        <v>1.379310344827589E-2</v>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="D1:D1048576">
+    <cfRule type="colorScale" priority="3">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H2:H8">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L2:L8">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{09FDD1CC-9ED4-4593-9CF0-ACFF7E44F672}">
+  <dimension ref="A1:L8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.140625" customWidth="1"/>
-    <col min="6" max="6" width="8.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.5703125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="14" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="14" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14" style="3" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14.28515625" style="3" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.42578125" style="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="J1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>9</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>12</v>
       </c>
       <c r="B2">
         <v>100</v>
       </c>
       <c r="C2">
-        <v>2252</v>
+        <v>70.688999999999993</v>
       </c>
       <c r="D2">
-        <v>0</v>
-      </c>
-      <c r="E2" s="2">
-        <f t="shared" ref="E2:E3" si="0">D2/C2</f>
-        <v>0</v>
+        <v>1390</v>
+      </c>
+      <c r="E2">
+        <v>96.58</v>
       </c>
       <c r="F2">
-        <v>71.816000000000003</v>
+        <v>1560</v>
       </c>
       <c r="G2">
-        <v>1360</v>
+        <v>1440</v>
       </c>
       <c r="H2">
-        <v>113.15</v>
-      </c>
-      <c r="I2">
-        <v>2520</v>
-      </c>
-      <c r="J2">
-        <v>1430</v>
-      </c>
-      <c r="K2">
-        <v>1490</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+        <v>1460</v>
+      </c>
+      <c r="I2" s="3">
+        <f>'1.0.31-cjs'!C2/'1.0.31-rrst'!C2</f>
+        <v>1.0159430745943501</v>
+      </c>
+      <c r="J2" s="3">
+        <f>'1.0.31-rrst'!D2/'1.0.31-cjs'!D2</f>
+        <v>1.0220588235294117</v>
+      </c>
+      <c r="K2" s="3">
+        <f>'1.0.31-rrst'!E2/'1.0.31-cjs'!E2</f>
+        <v>0.85355722492266894</v>
+      </c>
+      <c r="L2" s="3">
+        <f>'1.0.31-rrst'!F2/'1.0.31-cjs'!F2</f>
+        <v>0.61904761904761907</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B3">
         <v>100</v>
       </c>
       <c r="C3">
-        <v>61821</v>
+        <v>3673.1170000000002</v>
       </c>
       <c r="D3">
-        <v>0</v>
-      </c>
-      <c r="E3" s="2">
-        <f t="shared" si="0"/>
-        <v>0</v>
+        <v>27.21</v>
+      </c>
+      <c r="E3">
+        <v>9.18</v>
       </c>
       <c r="F3">
-        <v>2058.9180000000001</v>
+        <v>109.02</v>
       </c>
       <c r="G3">
-        <v>48.53</v>
+        <v>36.130000000000003</v>
       </c>
       <c r="H3">
-        <v>18.29</v>
-      </c>
-      <c r="I3">
-        <v>572.87</v>
-      </c>
-      <c r="J3">
-        <v>62.05</v>
-      </c>
-      <c r="K3">
-        <v>65.72</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+        <v>37.97</v>
+      </c>
+      <c r="I3" s="3">
+        <f>'1.0.31-cjs'!C3/'1.0.31-rrst'!C3</f>
+        <v>0.56053700440252785</v>
+      </c>
+      <c r="J3" s="3">
+        <f>'1.0.31-rrst'!D3/'1.0.31-cjs'!D3</f>
+        <v>0.56068411291984344</v>
+      </c>
+      <c r="K3" s="3">
+        <f>'1.0.31-rrst'!E3/'1.0.31-cjs'!E3</f>
+        <v>0.50191361399671952</v>
+      </c>
+      <c r="L3" s="3">
+        <f>'1.0.31-rrst'!F3/'1.0.31-cjs'!F3</f>
+        <v>0.19030495574912282</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B4">
         <v>100</v>
       </c>
       <c r="C4">
-        <v>177268</v>
+        <v>9494.1419999999998</v>
       </c>
       <c r="D4">
-        <v>0</v>
-      </c>
-      <c r="E4" s="2">
-        <f>D4/C4</f>
-        <v>0</v>
+        <v>10.52</v>
+      </c>
+      <c r="E4">
+        <v>0.55889999999999995</v>
       </c>
       <c r="F4">
-        <v>5905.6930000000002</v>
+        <v>47.34</v>
       </c>
       <c r="G4">
-        <v>16.920000000000002</v>
+        <v>14.62</v>
       </c>
       <c r="H4">
-        <v>2.83</v>
-      </c>
-      <c r="I4">
-        <v>255.29</v>
-      </c>
-      <c r="J4">
-        <v>23.13</v>
-      </c>
-      <c r="K4">
-        <v>24.24</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+        <v>16.100000000000001</v>
+      </c>
+      <c r="I4" s="3">
+        <f>'1.0.31-cjs'!C4/'1.0.31-rrst'!C4</f>
+        <v>0.62203546144559463</v>
+      </c>
+      <c r="J4" s="3">
+        <f>'1.0.31-rrst'!D4/'1.0.31-cjs'!D4</f>
+        <v>0.62174940898345143</v>
+      </c>
+      <c r="K4" s="3">
+        <f>'1.0.31-rrst'!E4/'1.0.31-cjs'!E4</f>
+        <v>0.19749116607773851</v>
+      </c>
+      <c r="L4" s="3">
+        <f>'1.0.31-rrst'!F4/'1.0.31-cjs'!F4</f>
+        <v>0.18543617062948023</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B5">
         <v>100</v>
       </c>
       <c r="C5">
-        <v>75710</v>
+        <v>4125.4129999999996</v>
       </c>
       <c r="D5">
-        <v>0</v>
-      </c>
-      <c r="E5" s="2">
-        <f>D5/C5</f>
-        <v>0</v>
+        <v>24.22</v>
+      </c>
+      <c r="E5">
+        <v>3.4</v>
       </c>
       <c r="F5">
-        <v>2520.547</v>
+        <v>79.069999999999993</v>
       </c>
       <c r="G5">
-        <v>39.64</v>
+        <v>38.049999999999997</v>
       </c>
       <c r="H5">
-        <v>3.95</v>
-      </c>
-      <c r="I5">
-        <v>1050</v>
-      </c>
-      <c r="J5">
-        <v>42.44</v>
-      </c>
-      <c r="K5">
-        <v>43.81</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+        <v>41.97</v>
+      </c>
+      <c r="I5" s="3">
+        <f>'1.0.31-cjs'!C5/'1.0.31-rrst'!C5</f>
+        <v>0.6109805248589657</v>
+      </c>
+      <c r="J5" s="3">
+        <f>'1.0.31-rrst'!D5/'1.0.31-cjs'!D5</f>
+        <v>0.61099899091826437</v>
+      </c>
+      <c r="K5" s="3">
+        <f>'1.0.31-rrst'!E5/'1.0.31-cjs'!E5</f>
+        <v>0.860759493670886</v>
+      </c>
+      <c r="L5" s="3">
+        <f>'1.0.31-rrst'!F5/'1.0.31-cjs'!F5</f>
+        <v>7.5304761904761902E-2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B6">
         <v>100</v>
       </c>
       <c r="C6">
-        <v>5717</v>
+        <v>217.511</v>
       </c>
       <c r="D6">
-        <v>0</v>
-      </c>
-      <c r="E6" s="2">
-        <f>D6/C6</f>
-        <v>0</v>
+        <v>457.99</v>
+      </c>
+      <c r="E6">
+        <v>10.91</v>
       </c>
       <c r="F6">
-        <v>187.39500000000001</v>
+        <v>982.03</v>
       </c>
       <c r="G6">
-        <v>529.26</v>
+        <v>474.76</v>
       </c>
       <c r="H6">
-        <v>25.42</v>
-      </c>
-      <c r="I6">
-        <v>13540</v>
-      </c>
-      <c r="J6">
-        <v>585.67999999999995</v>
-      </c>
-      <c r="K6">
-        <v>622.70000000000005</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+        <v>484.99</v>
+      </c>
+      <c r="I6" s="3">
+        <f>'1.0.31-cjs'!C6/'1.0.31-rrst'!C6</f>
+        <v>0.86154263462537528</v>
+      </c>
+      <c r="J6" s="3">
+        <f>'1.0.31-rrst'!D6/'1.0.31-cjs'!D6</f>
+        <v>0.86534028643766769</v>
+      </c>
+      <c r="K6" s="3">
+        <f>'1.0.31-rrst'!E6/'1.0.31-cjs'!E6</f>
+        <v>0.42918961447678988</v>
+      </c>
+      <c r="L6" s="3">
+        <f>'1.0.31-rrst'!F6/'1.0.31-cjs'!F6</f>
+        <v>7.252806499261448E-2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="B7">
         <v>100</v>
       </c>
       <c r="C7">
-        <v>122839</v>
+        <v>7643.0460000000003</v>
       </c>
       <c r="D7">
-        <v>0</v>
-      </c>
-      <c r="E7" s="2">
-        <f>D7/C7</f>
-        <v>0</v>
+        <v>13.07</v>
+      </c>
+      <c r="E7">
+        <v>2.0499999999999998</v>
       </c>
       <c r="F7">
-        <v>4093.308</v>
+        <v>92.06</v>
       </c>
       <c r="G7">
-        <v>24.41</v>
+        <v>17.63</v>
       </c>
       <c r="H7">
-        <v>5.76</v>
-      </c>
-      <c r="I7">
-        <v>351.38</v>
-      </c>
-      <c r="J7">
-        <v>30.24</v>
-      </c>
-      <c r="K7">
-        <v>33.46</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+        <v>19.28</v>
+      </c>
+      <c r="I7" s="3">
+        <f>'1.0.31-cjs'!C7/'1.0.31-rrst'!C7</f>
+        <v>0.53555977551358447</v>
+      </c>
+      <c r="J7" s="3">
+        <f>'1.0.31-rrst'!D7/'1.0.31-cjs'!D7</f>
+        <v>0.53543629659975422</v>
+      </c>
+      <c r="K7" s="3">
+        <f>'1.0.31-rrst'!E7/'1.0.31-cjs'!E7</f>
+        <v>0.35590277777777773</v>
+      </c>
+      <c r="L7" s="3">
+        <f>'1.0.31-rrst'!F7/'1.0.31-cjs'!F7</f>
+        <v>0.26199556036200128</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B8">
         <v>100</v>
       </c>
       <c r="C8">
-        <v>2201</v>
+        <v>70.218999999999994</v>
       </c>
       <c r="D8">
+        <v>1400</v>
+      </c>
+      <c r="E8">
+        <v>94.8</v>
+      </c>
+      <c r="F8">
+        <v>1480</v>
+      </c>
+      <c r="G8">
+        <v>1440</v>
+      </c>
+      <c r="H8">
+        <v>1450</v>
+      </c>
+      <c r="I8" s="3">
+        <f>'1.0.31-cjs'!C8/'1.0.31-rrst'!C8</f>
+        <v>0.99868981329839501</v>
+      </c>
+      <c r="J8" s="3">
+        <f>'1.0.31-rrst'!D8/'1.0.31-cjs'!D8</f>
+        <v>1.0071942446043165</v>
+      </c>
+      <c r="K8" s="3">
+        <f>'1.0.31-rrst'!E8/'1.0.31-cjs'!E8</f>
+        <v>0.70446607713457676</v>
+      </c>
+      <c r="L8" s="3">
+        <f>'1.0.31-rrst'!F8/'1.0.31-cjs'!F8</f>
+        <v>0.75126903553299496</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{059A8E8E-4130-4CCA-A3A8-A42D26512C95}">
+  <dimension ref="A1:H8"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14.28515625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="E8" s="2">
-        <f>D8/C8</f>
-        <v>0</v>
+      <c r="B1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2">
+        <v>100</v>
+      </c>
+      <c r="C2">
+        <v>71.816000000000003</v>
+      </c>
+      <c r="D2">
+        <v>1360</v>
+      </c>
+      <c r="E2">
+        <v>113.15</v>
+      </c>
+      <c r="F2">
+        <v>2520</v>
+      </c>
+      <c r="G2">
+        <v>1430</v>
+      </c>
+      <c r="H2">
+        <v>1490</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3">
+        <v>100</v>
+      </c>
+      <c r="C3">
+        <v>2058.9180000000001</v>
+      </c>
+      <c r="D3">
+        <v>48.53</v>
+      </c>
+      <c r="E3">
+        <v>18.29</v>
+      </c>
+      <c r="F3">
+        <v>572.87</v>
+      </c>
+      <c r="G3">
+        <v>62.05</v>
+      </c>
+      <c r="H3">
+        <v>65.72</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4">
+        <v>100</v>
+      </c>
+      <c r="C4">
+        <v>5905.6930000000002</v>
+      </c>
+      <c r="D4">
+        <v>16.920000000000002</v>
+      </c>
+      <c r="E4">
+        <v>2.83</v>
+      </c>
+      <c r="F4">
+        <v>255.29</v>
+      </c>
+      <c r="G4">
+        <v>23.13</v>
+      </c>
+      <c r="H4">
+        <v>24.24</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5">
+        <v>100</v>
+      </c>
+      <c r="C5">
+        <v>2520.547</v>
+      </c>
+      <c r="D5">
+        <v>39.64</v>
+      </c>
+      <c r="E5">
+        <v>3.95</v>
+      </c>
+      <c r="F5">
+        <v>1050</v>
+      </c>
+      <c r="G5">
+        <v>42.44</v>
+      </c>
+      <c r="H5">
+        <v>43.81</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6">
+        <v>100</v>
+      </c>
+      <c r="C6">
+        <v>187.39500000000001</v>
+      </c>
+      <c r="D6">
+        <v>529.26</v>
+      </c>
+      <c r="E6">
+        <v>25.42</v>
+      </c>
+      <c r="F6">
+        <v>13540</v>
+      </c>
+      <c r="G6">
+        <v>585.67999999999995</v>
+      </c>
+      <c r="H6">
+        <v>622.70000000000005</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7">
+        <v>100</v>
+      </c>
+      <c r="C7">
+        <v>4093.308</v>
+      </c>
+      <c r="D7">
+        <v>24.41</v>
+      </c>
+      <c r="E7">
+        <v>5.76</v>
+      </c>
+      <c r="F7">
+        <v>351.38</v>
+      </c>
+      <c r="G7">
+        <v>30.24</v>
+      </c>
+      <c r="H7">
+        <v>33.46</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8">
+        <v>100</v>
+      </c>
+      <c r="C8">
+        <v>70.126999999999995</v>
+      </c>
+      <c r="D8">
+        <v>1390</v>
+      </c>
+      <c r="E8">
+        <v>134.57</v>
       </c>
       <c r="F8">
-        <v>70.126999999999995</v>
+        <v>1970</v>
       </c>
       <c r="G8">
-        <v>1390</v>
+        <v>1450</v>
       </c>
       <c r="H8">
-        <v>134.57</v>
-      </c>
-      <c r="I8">
-        <v>1970</v>
-      </c>
-      <c r="J8">
-        <v>1450</v>
-      </c>
-      <c r="K8">
         <v>1470</v>
       </c>
     </row>

</xml_diff>